<commit_message>
Update Spain CPI data
Refresh the Spain CPI Excel dataset in Data/Spain/CPI.xlsx with the latest available inflation values to keep the time series current.
</commit_message>
<xml_diff>
--- a/Data/Spain/CPI.xlsx
+++ b/Data/Spain/CPI.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\noboy\Repos\eu-sae-personal\Data\Spain\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F25E5289-4D79-4C5D-B814-1BEAA836C175}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12D7ECE6-C315-4C91-A84A-B93393A9336D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{698DB3C2-4DC5-4715-8721-3BA626112B86}"/>
+    <workbookView xWindow="4800" yWindow="3110" windowWidth="14400" windowHeight="8170" xr2:uid="{698DB3C2-4DC5-4715-8721-3BA626112B86}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -416,7 +416,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEC33518-48A4-4A87-8F67-F72B8FF6AB40}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
@@ -429,17 +429,25 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2">
-        <v>2012</v>
+        <v>2011</v>
       </c>
       <c r="B2">
-        <v>120</v>
+        <v>110</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3">
+        <v>2012</v>
+      </c>
+      <c r="B3">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4">
         <v>2013</v>
       </c>
-      <c r="B3">
+      <c r="B4">
         <v>130</v>
       </c>
     </row>

</xml_diff>